<commit_message>
Actualizar maestro Falabella con nuevos productos
</commit_message>
<xml_diff>
--- a/public/falabella-productos.xlsx
+++ b/public/falabella-productos.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Productos Falabella" sheetId="2" r:id="R25d714532aee438d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Productos Falabella" sheetId="2" r:id="R75a2f75f496d41da"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -43,7 +43,7 @@
       <x:name val="Arial"/>
     </x:font>
   </x:fonts>
-  <x:fills count="6">
+  <x:fills count="7">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -70,6 +70,11 @@
         <x:fgColor rgb="FF0F766E"/>
       </x:patternFill>
     </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF0F766E"/>
+      </x:patternFill>
+    </x:fill>
   </x:fills>
   <x:borders count="2">
     <x:border/>
@@ -82,7 +87,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="24">
+  <x:cellXfs count="30">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <x:xf numFmtId="49" fontId="1" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -137,6 +142,24 @@
       <x:alignment horizontal="center" vertical="center" wrapText="1"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="2" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="49" fontId="3" fillId="6" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="6" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="49" fontId="2" fillId="6" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="2" fillId="6" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="2" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="center" vertical="center"/>
     </x:xf>
   </x:cellXfs>
@@ -369,28 +392,28 @@
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="24" customHeight="1">
-      <x:c r="A1" s="21" t="str">
+      <x:c r="A1" s="27" t="str">
         <x:v>SellerSku</x:v>
       </x:c>
-      <x:c r="B1" s="21" t="str">
+      <x:c r="B1" s="27" t="str">
         <x:v>ShopSku</x:v>
       </x:c>
-      <x:c r="C1" s="22" t="str">
+      <x:c r="C1" s="28" t="str">
         <x:v>Name</x:v>
       </x:c>
-      <x:c r="D1" s="22" t="str">
+      <x:c r="D1" s="28" t="str">
         <x:v>ProductData.Sabor</x:v>
       </x:c>
-      <x:c r="E1" s="22" t="str">
+      <x:c r="E1" s="28" t="str">
         <x:v>ProductData.Model</x:v>
       </x:c>
-      <x:c r="F1" s="22" t="str">
+      <x:c r="F1" s="28" t="str">
         <x:v>Variation</x:v>
       </x:c>
-      <x:c r="G1" s="23" t="str">
+      <x:c r="G1" s="29" t="str">
         <x:v>Columna1</x:v>
       </x:c>
-      <x:c r="H1" s="23" t="str">
+      <x:c r="H1" s="29" t="str">
         <x:v>SaborVariant</x:v>
       </x:c>
     </x:row>
@@ -50728,6 +50751,366 @@
         <x:v>Otro Sabor</x:v>
       </x:c>
     </x:row>
+    <x:row r="2260">
+      <x:c r="A2260" s="16" t="str">
+        <x:v>APN53</x:v>
+      </x:c>
+      <x:c r="B2260" s="16" t="str">
+        <x:v>158827818</x:v>
+      </x:c>
+      <x:c r="C2260" s="17" t="str">
+        <x:v>PROTEINA CRITICAL WHEY 132GR 4SV CHOCOLATE MILKSHAKE- APPLIED NUTRITION</x:v>
+      </x:c>
+      <x:c r="D2260" s="17" t="str"/>
+      <x:c r="E2260" s="17" t="str"/>
+      <x:c r="F2260" s="17" t="str"/>
+      <x:c r="G2260" s="17" t="str">
+        <x:v>PROTEINA CRITICAL WHEY 132GR 4SV CHOCOLATE MILKSHAKE- APPLIED NUTRITION</x:v>
+      </x:c>
+      <x:c r="H2260" s="17" t="str">
+        <x:v>Chocolate</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="2261">
+      <x:c r="A2261" s="16" t="str">
+        <x:v>APN67</x:v>
+      </x:c>
+      <x:c r="B2261" s="16" t="str">
+        <x:v>158828110</x:v>
+      </x:c>
+      <x:c r="C2261" s="17" t="str">
+        <x:v>SHAKER TAPA AZUL 700ML- APPLIED NUTRITION</x:v>
+      </x:c>
+      <x:c r="D2261" s="17" t="str"/>
+      <x:c r="E2261" s="17" t="str"/>
+      <x:c r="F2261" s="17" t="str">
+        <x:v>...</x:v>
+      </x:c>
+      <x:c r="G2261" s="17" t="str">
+        <x:v>SHAKER TAPA AZUL 700ML- APPLIED NUTRITION</x:v>
+      </x:c>
+      <x:c r="H2261" s="17" t="str"/>
+    </x:row>
+    <x:row r="2262">
+      <x:c r="A2262" s="16" t="str">
+        <x:v>OST211</x:v>
+      </x:c>
+      <x:c r="B2262" s="16" t="str">
+        <x:v>158830019</x:v>
+      </x:c>
+      <x:c r="C2262" s="17" t="str">
+        <x:v>SHAKER  BLANCO CON MORADO 700ML  - OSTROVIT</x:v>
+      </x:c>
+      <x:c r="D2262" s="17" t="str"/>
+      <x:c r="E2262" s="17" t="str"/>
+      <x:c r="F2262" s="17" t="str">
+        <x:v>...</x:v>
+      </x:c>
+      <x:c r="G2262" s="17" t="str">
+        <x:v>SHAKER  BLANCO CON MORADO 700ML  - OSTROVIT</x:v>
+      </x:c>
+      <x:c r="H2262" s="17" t="str"/>
+    </x:row>
+    <x:row r="2263">
+      <x:c r="A2263" s="16" t="str">
+        <x:v>APN54</x:v>
+      </x:c>
+      <x:c r="B2263" s="16" t="str">
+        <x:v>158833248</x:v>
+      </x:c>
+      <x:c r="C2263" s="17" t="str">
+        <x:v>PROTEINA CRITICAL WHEY 825GR 25SV - APPLIED NUTRITION</x:v>
+      </x:c>
+      <x:c r="D2263" s="17" t="str"/>
+      <x:c r="E2263" s="17" t="str"/>
+      <x:c r="F2263" s="17" t="str"/>
+      <x:c r="G2263" s="17" t="str">
+        <x:v>PROTEINA CRITICAL WHEY 825GR 25SV - APPLIED NUTRITION - Otro Sabor</x:v>
+      </x:c>
+      <x:c r="H2263" s="17" t="str">
+        <x:v>Otro Sabor</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="2264">
+      <x:c r="A2264" s="16" t="str">
+        <x:v>APN55</x:v>
+      </x:c>
+      <x:c r="B2264" s="16" t="str">
+        <x:v>158833247</x:v>
+      </x:c>
+      <x:c r="C2264" s="17" t="str">
+        <x:v>PROTEINA CRITICAL WHEY 825GR 25SV - APPLIED NUTRITION</x:v>
+      </x:c>
+      <x:c r="D2264" s="17" t="str"/>
+      <x:c r="E2264" s="17" t="str"/>
+      <x:c r="F2264" s="17" t="str"/>
+      <x:c r="G2264" s="17" t="str">
+        <x:v>PROTEINA CRITICAL WHEY 825GR 25SV - APPLIED NUTRITION - Banana</x:v>
+      </x:c>
+      <x:c r="H2264" s="17" t="str">
+        <x:v>Banana</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="2265">
+      <x:c r="A2265" s="16" t="str">
+        <x:v>APN56</x:v>
+      </x:c>
+      <x:c r="B2265" s="16" t="str">
+        <x:v>158833246</x:v>
+      </x:c>
+      <x:c r="C2265" s="17" t="str">
+        <x:v>PROTEINA CRITICAL WHEY 825GR 25SV - APPLIED NUTRITION</x:v>
+      </x:c>
+      <x:c r="D2265" s="17" t="str"/>
+      <x:c r="E2265" s="17" t="str"/>
+      <x:c r="F2265" s="17" t="str"/>
+      <x:c r="G2265" s="17" t="str">
+        <x:v>PROTEINA CRITICAL WHEY 825GR 25SV - APPLIED NUTRITION - Frutilla</x:v>
+      </x:c>
+      <x:c r="H2265" s="17" t="str">
+        <x:v>Frutilla</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="2266">
+      <x:c r="A2266" s="16" t="str">
+        <x:v>APN57</x:v>
+      </x:c>
+      <x:c r="B2266" s="16" t="str">
+        <x:v>158833245</x:v>
+      </x:c>
+      <x:c r="C2266" s="17" t="str">
+        <x:v>PROTEINA CRITICAL WHEY 825GR 25SV - APPLIED NUTRITION</x:v>
+      </x:c>
+      <x:c r="D2266" s="17" t="str"/>
+      <x:c r="E2266" s="17" t="str"/>
+      <x:c r="F2266" s="17" t="str"/>
+      <x:c r="G2266" s="17" t="str">
+        <x:v>PROTEINA CRITICAL WHEY 825GR 25SV - APPLIED NUTRITION - Salted Caramel</x:v>
+      </x:c>
+      <x:c r="H2266" s="17" t="str">
+        <x:v>Salted Caramel</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="2267">
+      <x:c r="A2267" s="16" t="str">
+        <x:v>APN58</x:v>
+      </x:c>
+      <x:c r="B2267" s="16" t="str">
+        <x:v>158833244</x:v>
+      </x:c>
+      <x:c r="C2267" s="17" t="str">
+        <x:v>PROTEINA CRITICAL WHEY 825GR 25SV - APPLIED NUTRITION</x:v>
+      </x:c>
+      <x:c r="D2267" s="17" t="str"/>
+      <x:c r="E2267" s="17" t="str"/>
+      <x:c r="F2267" s="17" t="str"/>
+      <x:c r="G2267" s="17" t="str">
+        <x:v>PROTEINA CRITICAL WHEY 825GR 25SV - APPLIED NUTRITION - Chocolate</x:v>
+      </x:c>
+      <x:c r="H2267" s="17" t="str">
+        <x:v>Chocolate</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="2268">
+      <x:c r="A2268" s="16" t="str">
+        <x:v>APN59</x:v>
+      </x:c>
+      <x:c r="B2268" s="16" t="str">
+        <x:v>158833243</x:v>
+      </x:c>
+      <x:c r="C2268" s="17" t="str">
+        <x:v>PROTEINA CRITICAL WHEY 825GR 25SV - APPLIED NUTRITION</x:v>
+      </x:c>
+      <x:c r="D2268" s="17" t="str"/>
+      <x:c r="E2268" s="17" t="str"/>
+      <x:c r="F2268" s="17" t="str"/>
+      <x:c r="G2268" s="17" t="str">
+        <x:v>PROTEINA CRITICAL WHEY 825GR 25SV - APPLIED NUTRITION - Vainilla</x:v>
+      </x:c>
+      <x:c r="H2268" s="17" t="str">
+        <x:v>Vainilla</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="2269">
+      <x:c r="A2269" s="16" t="str">
+        <x:v>APN60</x:v>
+      </x:c>
+      <x:c r="B2269" s="16" t="str">
+        <x:v>158833242</x:v>
+      </x:c>
+      <x:c r="C2269" s="17" t="str">
+        <x:v>PROTEINA CRITICAL WHEY 825GR 25SV - APPLIED NUTRITION</x:v>
+      </x:c>
+      <x:c r="D2269" s="17" t="str"/>
+      <x:c r="E2269" s="17" t="str"/>
+      <x:c r="F2269" s="17" t="str"/>
+      <x:c r="G2269" s="17" t="str">
+        <x:v>PROTEINA CRITICAL WHEY 825GR 25SV - APPLIED NUTRITION - Caramelo</x:v>
+      </x:c>
+      <x:c r="H2269" s="17" t="str">
+        <x:v>Caramelo</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="2270">
+      <x:c r="A2270" s="16" t="str">
+        <x:v>APN61</x:v>
+      </x:c>
+      <x:c r="B2270" s="16" t="str">
+        <x:v>158833241</x:v>
+      </x:c>
+      <x:c r="C2270" s="17" t="str">
+        <x:v>PROTEINA CRITICAL WHEY 825GR 25SV - APPLIED NUTRITION</x:v>
+      </x:c>
+      <x:c r="D2270" s="17" t="str"/>
+      <x:c r="E2270" s="17" t="str"/>
+      <x:c r="F2270" s="17" t="str"/>
+      <x:c r="G2270" s="17" t="str">
+        <x:v>PROTEINA CRITICAL WHEY 825GR 25SV - APPLIED NUTRITION</x:v>
+      </x:c>
+      <x:c r="H2270" s="17" t="str">
+        <x:v>...</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="2271">
+      <x:c r="A2271" s="16" t="str">
+        <x:v>APN62</x:v>
+      </x:c>
+      <x:c r="B2271" s="16" t="str">
+        <x:v>158833240</x:v>
+      </x:c>
+      <x:c r="C2271" s="17" t="str">
+        <x:v>PROTEINA CRITICAL WHEY 825GR 25SV - APPLIED NUTRITION</x:v>
+      </x:c>
+      <x:c r="D2271" s="17" t="str"/>
+      <x:c r="E2271" s="17" t="str"/>
+      <x:c r="F2271" s="17" t="str"/>
+      <x:c r="G2271" s="17" t="str">
+        <x:v>PROTEINA CRITICAL WHEY 825GR 25SV - APPLIED NUTRITION - Chocolate Blanco</x:v>
+      </x:c>
+      <x:c r="H2271" s="17" t="str">
+        <x:v>Chocolate Blanco</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="2272">
+      <x:c r="A2272" s="16" t="str">
+        <x:v>APN63</x:v>
+      </x:c>
+      <x:c r="B2272" s="16" t="str">
+        <x:v>158833239</x:v>
+      </x:c>
+      <x:c r="C2272" s="17" t="str">
+        <x:v>PROTEINA CRITICAL WHEY 825GR 25SV - APPLIED NUTRITION</x:v>
+      </x:c>
+      <x:c r="D2272" s="17" t="str"/>
+      <x:c r="E2272" s="17" t="str"/>
+      <x:c r="F2272" s="17" t="str"/>
+      <x:c r="G2272" s="17" t="str">
+        <x:v>PROTEINA CRITICAL WHEY 825GR 25SV - APPLIED NUTRITION - Vainilla Ice Cream</x:v>
+      </x:c>
+      <x:c r="H2272" s="17" t="str">
+        <x:v>Vainilla Ice Cream</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="2273">
+      <x:c r="A2273" s="16" t="str">
+        <x:v>APN64</x:v>
+      </x:c>
+      <x:c r="B2273" s="16" t="str">
+        <x:v>158833238</x:v>
+      </x:c>
+      <x:c r="C2273" s="17" t="str">
+        <x:v>PROTEINA CRITICAL WHEY 825GR 25SV - APPLIED NUTRITION</x:v>
+      </x:c>
+      <x:c r="D2273" s="17" t="str"/>
+      <x:c r="E2273" s="17" t="str"/>
+      <x:c r="F2273" s="17" t="str"/>
+      <x:c r="G2273" s="17" t="str">
+        <x:v>PROTEINA CRITICAL WHEY 825GR 25SV - APPLIED NUTRITION - Pistacho</x:v>
+      </x:c>
+      <x:c r="H2273" s="17" t="str">
+        <x:v>Pistacho</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="2274">
+      <x:c r="A2274" s="16" t="str">
+        <x:v>APN65</x:v>
+      </x:c>
+      <x:c r="B2274" s="16" t="str">
+        <x:v>158833237</x:v>
+      </x:c>
+      <x:c r="C2274" s="17" t="str">
+        <x:v>PROTEINA CRITICAL WHEY 825GR 25SV - APPLIED NUTRITION</x:v>
+      </x:c>
+      <x:c r="D2274" s="17" t="str"/>
+      <x:c r="E2274" s="17" t="str"/>
+      <x:c r="F2274" s="17" t="str"/>
+      <x:c r="G2274" s="17" t="str">
+        <x:v>PROTEINA CRITICAL WHEY 825GR 25SV - APPLIED NUTRITION - Cookies and Cream</x:v>
+      </x:c>
+      <x:c r="H2274" s="17" t="str">
+        <x:v>Cookies and Cream</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="2275">
+      <x:c r="A2275" s="16" t="str">
+        <x:v>APN66</x:v>
+      </x:c>
+      <x:c r="B2275" s="16" t="str">
+        <x:v>158833236</x:v>
+      </x:c>
+      <x:c r="C2275" s="17" t="str">
+        <x:v>PROTEINA CRITICAL WHEY 825GR 25SV - APPLIED NUTRITION</x:v>
+      </x:c>
+      <x:c r="D2275" s="17" t="str"/>
+      <x:c r="E2275" s="17" t="str"/>
+      <x:c r="F2275" s="17" t="str"/>
+      <x:c r="G2275" s="17" t="str">
+        <x:v>PROTEINA CRITICAL WHEY 825GR 25SV - APPLIED NUTRITION - Almendra</x:v>
+      </x:c>
+      <x:c r="H2275" s="17" t="str">
+        <x:v>Almendra</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="2276">
+      <x:c r="A2276" s="16" t="str">
+        <x:v>ORX46</x:v>
+      </x:c>
+      <x:c r="B2276" s="16" t="str">
+        <x:v>158836574</x:v>
+      </x:c>
+      <x:c r="C2276" s="17" t="str">
+        <x:v>PACK BANDA ELÁSTICA-GUANTES GRAB-BANDA RESISTENCIA NEGRO- ORXFIT</x:v>
+      </x:c>
+      <x:c r="D2276" s="17" t="str"/>
+      <x:c r="E2276" s="17" t="str"/>
+      <x:c r="F2276" s="17" t="str">
+        <x:v>...</x:v>
+      </x:c>
+      <x:c r="G2276" s="17" t="str">
+        <x:v>PACK BANDA ELÁSTICA-GUANTES GRAB-BANDA RESISTENCIA NEGRO- ORXFIT</x:v>
+      </x:c>
+      <x:c r="H2276" s="17" t="str"/>
+    </x:row>
+    <x:row r="2277">
+      <x:c r="A2277" s="16" t="str">
+        <x:v>BOX-09</x:v>
+      </x:c>
+      <x:c r="B2277" s="16" t="str">
+        <x:v>158839641</x:v>
+      </x:c>
+      <x:c r="C2277" s="17" t="str">
+        <x:v>Box 12 barras de proteina 60GR C/U CHOCOLATE FUDGE - SLIMBAR</x:v>
+      </x:c>
+      <x:c r="D2277" s="17" t="str"/>
+      <x:c r="E2277" s="17" t="str"/>
+      <x:c r="F2277" s="17" t="str"/>
+      <x:c r="G2277" s="17" t="str">
+        <x:v>Box 12 barras de proteina 60GR C/U CHOCOLATE FUDGE - SLIMBAR</x:v>
+      </x:c>
+      <x:c r="H2277" s="17" t="str">
+        <x:v>Chocolate</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>

</xml_diff>